<commit_message>
1.5.0: add_to_tracker.py adds every qualifying job; Assistant Notes column keeps Notes for the person; review pass in the AI guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015QuzxbVg7RLWTYXhDF5qUn
</commit_message>
<xml_diff>
--- a/templates/job_tracker_template.xlsx
+++ b/templates/job_tracker_template.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2000"/>
+  <dimension ref="A1:O2000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -528,6 +529,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Assistant Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -10544,7 +10550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -10557,9 +10563,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -10596,34 +10600,44 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Notes: yours. Your assistant never writes here; it reads your notes to learn what to change in your search.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>After adding rows, run: python3 tools/import_tracker.py path/to/this/file.xlsx</t>
+          <t>Assistant Notes: your assistant's match rationale and flags for each job.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>That keeps tracked jobs from showing up again and adds new companies to search.</t>
-        </is>
-      </c>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>To add the pipeline's shortlist here: run python3 tools/export_shortlist.py and paste rows from the CSV in exports/.</t>
+          <t>Daily: python3 tools/add_to_tracker.py adds every qualifying job here with Status New.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Review the New rows: set Status (Applied, Did Not Apply, ...) and write your reasons in Notes.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>Added rows by hand? Run python3 tools/import_tracker.py path/to/this/file.xlsx so those jobs don't come back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>You can rename or add columns. If you rename Company, Job Title, Status or Link, update config/tracker_map.json.</t>
         </is>

</xml_diff>